<commit_message>
update decision tables with cat 2 buffers
</commit_message>
<xml_diff>
--- a/Document/report/Decision Table/Decision Table.xlsx
+++ b/Document/report/Decision Table/Decision Table.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason.Cope\Documents\Current Action\Assessments\Rougheye_blackspotted_2025\STAR requests\Request 13\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason.Cope\Documents\Github\REBS-2025\Document\report\Decision Table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF0C18D1-FF09-4736-9CB4-EB70984299AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B566204-D27D-41B6-8B83-2F77B38519EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{505FE161-4ED4-4F9D-B2FA-1BF4DC518013}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
+    <sheet name="Tables" sheetId="3" r:id="rId1"/>
+    <sheet name="Cat 1" sheetId="4" r:id="rId2"/>
+    <sheet name="Cat 2" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="19">
   <si>
     <t>Year</t>
   </si>
@@ -209,6 +213,15 @@
       </rPr>
       <t>=0.039</t>
     </r>
+  </si>
+  <si>
+    <t>Cat 1</t>
+  </si>
+  <si>
+    <t>Cat2</t>
+  </si>
+  <si>
+    <t>Projections use 2026 fleet allocations</t>
   </si>
 </sst>
 </file>
@@ -547,28 +560,6 @@
     <xf numFmtId="4" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -584,14 +575,8 @@
     <xf numFmtId="165" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -618,6 +603,34 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -944,72 +957,72 @@
     <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="30"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="39"/>
-      <c r="T1" s="39"/>
-      <c r="U1" s="39"/>
-      <c r="V1" s="39"/>
-      <c r="W1" s="39"/>
-      <c r="X1" s="39"/>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="39"/>
-      <c r="AE1" s="39"/>
-      <c r="AF1" s="39"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="46"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
+      <c r="X1" s="28"/>
+      <c r="Y1" s="28"/>
+      <c r="Z1" s="28"/>
+      <c r="AA1" s="28"/>
+      <c r="AB1" s="28"/>
+      <c r="AC1" s="28"/>
+      <c r="AD1" s="28"/>
+      <c r="AE1" s="28"/>
+      <c r="AF1" s="28"/>
     </row>
     <row r="2" spans="1:32" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13"/>
       <c r="B2" s="12"/>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="23" t="s">
+      <c r="D2" s="47"/>
+      <c r="E2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="24"/>
-      <c r="G2" s="25" t="s">
+      <c r="F2" s="48"/>
+      <c r="G2" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="26"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="39"/>
-      <c r="V2" s="40"/>
-      <c r="W2" s="41"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="41"/>
-      <c r="Z2" s="41"/>
-      <c r="AA2" s="41"/>
-      <c r="AB2" s="41"/>
-      <c r="AC2" s="41"/>
-      <c r="AD2" s="41"/>
-      <c r="AE2" s="41"/>
-      <c r="AF2" s="39"/>
+      <c r="H2" s="50"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
+      <c r="S2" s="42"/>
+      <c r="T2" s="42"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="29"/>
+      <c r="W2" s="42"/>
+      <c r="X2" s="42"/>
+      <c r="Y2" s="42"/>
+      <c r="Z2" s="42"/>
+      <c r="AA2" s="42"/>
+      <c r="AB2" s="42"/>
+      <c r="AC2" s="42"/>
+      <c r="AD2" s="42"/>
+      <c r="AE2" s="42"/>
+      <c r="AF2" s="28"/>
     </row>
     <row r="3" spans="1:32" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -1036,28 +1049,28 @@
       <c r="H3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="42"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
-      <c r="O3" s="43"/>
-      <c r="P3" s="43"/>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="43"/>
-      <c r="S3" s="43"/>
-      <c r="T3" s="43"/>
-      <c r="U3" s="39"/>
-      <c r="V3" s="42"/>
-      <c r="W3" s="43"/>
-      <c r="X3" s="43"/>
-      <c r="Y3" s="43"/>
-      <c r="Z3" s="43"/>
-      <c r="AA3" s="43"/>
-      <c r="AB3" s="43"/>
-      <c r="AC3" s="43"/>
-      <c r="AD3" s="43"/>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="39"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="31"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="30"/>
+      <c r="W3" s="31"/>
+      <c r="X3" s="31"/>
+      <c r="Y3" s="31"/>
+      <c r="Z3" s="31"/>
+      <c r="AA3" s="31"/>
+      <c r="AB3" s="31"/>
+      <c r="AC3" s="31"/>
+      <c r="AD3" s="31"/>
+      <c r="AE3" s="31"/>
+      <c r="AF3" s="28"/>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A4" s="15">
@@ -1084,28 +1097,28 @@
       <c r="H4" s="10">
         <v>0.93285099999999999</v>
       </c>
-      <c r="K4" s="44"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="46"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="46"/>
-      <c r="Q4" s="47"/>
-      <c r="R4" s="47"/>
-      <c r="S4" s="46"/>
-      <c r="T4" s="47"/>
-      <c r="U4" s="39"/>
-      <c r="V4" s="44"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="46"/>
-      <c r="Y4" s="47"/>
-      <c r="Z4" s="48"/>
-      <c r="AA4" s="46"/>
-      <c r="AB4" s="47"/>
-      <c r="AC4" s="48"/>
-      <c r="AD4" s="46"/>
-      <c r="AE4" s="47"/>
-      <c r="AF4" s="39"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="34"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="34"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="28"/>
+      <c r="V4" s="32"/>
+      <c r="W4" s="33"/>
+      <c r="X4" s="34"/>
+      <c r="Y4" s="35"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="34"/>
+      <c r="AB4" s="35"/>
+      <c r="AC4" s="36"/>
+      <c r="AD4" s="34"/>
+      <c r="AE4" s="35"/>
+      <c r="AF4" s="28"/>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" s="16">
@@ -1132,28 +1145,28 @@
       <c r="H5" s="10">
         <v>0.93602700000000005</v>
       </c>
-      <c r="K5" s="44"/>
-      <c r="L5" s="45"/>
-      <c r="M5" s="46"/>
-      <c r="N5" s="47"/>
-      <c r="O5" s="47"/>
-      <c r="P5" s="46"/>
-      <c r="Q5" s="47"/>
-      <c r="R5" s="47"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="47"/>
-      <c r="U5" s="39"/>
-      <c r="V5" s="44"/>
-      <c r="W5" s="45"/>
-      <c r="X5" s="46"/>
-      <c r="Y5" s="47"/>
-      <c r="Z5" s="48"/>
-      <c r="AA5" s="46"/>
-      <c r="AB5" s="47"/>
-      <c r="AC5" s="48"/>
-      <c r="AD5" s="46"/>
-      <c r="AE5" s="47"/>
-      <c r="AF5" s="39"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="35"/>
+      <c r="O5" s="35"/>
+      <c r="P5" s="34"/>
+      <c r="Q5" s="35"/>
+      <c r="R5" s="35"/>
+      <c r="S5" s="34"/>
+      <c r="T5" s="35"/>
+      <c r="U5" s="28"/>
+      <c r="V5" s="32"/>
+      <c r="W5" s="33"/>
+      <c r="X5" s="34"/>
+      <c r="Y5" s="35"/>
+      <c r="Z5" s="36"/>
+      <c r="AA5" s="34"/>
+      <c r="AB5" s="35"/>
+      <c r="AC5" s="36"/>
+      <c r="AD5" s="34"/>
+      <c r="AE5" s="35"/>
+      <c r="AF5" s="28"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A6" s="16">
@@ -1180,28 +1193,28 @@
       <c r="H6" s="10">
         <v>0.93947000000000003</v>
       </c>
-      <c r="K6" s="44"/>
-      <c r="L6" s="49"/>
-      <c r="M6" s="46"/>
-      <c r="N6" s="47"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="46"/>
-      <c r="Q6" s="47"/>
-      <c r="R6" s="47"/>
-      <c r="S6" s="46"/>
-      <c r="T6" s="47"/>
-      <c r="U6" s="39"/>
-      <c r="V6" s="44"/>
-      <c r="W6" s="50"/>
-      <c r="X6" s="46"/>
-      <c r="Y6" s="47"/>
-      <c r="Z6" s="48"/>
-      <c r="AA6" s="46"/>
-      <c r="AB6" s="47"/>
-      <c r="AC6" s="48"/>
-      <c r="AD6" s="46"/>
-      <c r="AE6" s="47"/>
-      <c r="AF6" s="39"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="34"/>
+      <c r="N6" s="35"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="34"/>
+      <c r="Q6" s="35"/>
+      <c r="R6" s="35"/>
+      <c r="S6" s="34"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="28"/>
+      <c r="V6" s="32"/>
+      <c r="W6" s="38"/>
+      <c r="X6" s="34"/>
+      <c r="Y6" s="35"/>
+      <c r="Z6" s="36"/>
+      <c r="AA6" s="34"/>
+      <c r="AB6" s="35"/>
+      <c r="AC6" s="36"/>
+      <c r="AD6" s="34"/>
+      <c r="AE6" s="35"/>
+      <c r="AF6" s="28"/>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" s="16">
@@ -1228,28 +1241,28 @@
       <c r="H7" s="10">
         <v>0.94242599999999999</v>
       </c>
-      <c r="K7" s="44"/>
-      <c r="L7" s="49"/>
-      <c r="M7" s="46"/>
-      <c r="N7" s="47"/>
-      <c r="O7" s="47"/>
-      <c r="P7" s="46"/>
-      <c r="Q7" s="47"/>
-      <c r="R7" s="47"/>
-      <c r="S7" s="46"/>
-      <c r="T7" s="47"/>
-      <c r="U7" s="39"/>
-      <c r="V7" s="44"/>
-      <c r="W7" s="50"/>
-      <c r="X7" s="46"/>
-      <c r="Y7" s="47"/>
-      <c r="Z7" s="48"/>
-      <c r="AA7" s="46"/>
-      <c r="AB7" s="47"/>
-      <c r="AC7" s="48"/>
-      <c r="AD7" s="46"/>
-      <c r="AE7" s="47"/>
-      <c r="AF7" s="39"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="37"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="35"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="34"/>
+      <c r="Q7" s="35"/>
+      <c r="R7" s="35"/>
+      <c r="S7" s="34"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="28"/>
+      <c r="V7" s="32"/>
+      <c r="W7" s="38"/>
+      <c r="X7" s="34"/>
+      <c r="Y7" s="35"/>
+      <c r="Z7" s="36"/>
+      <c r="AA7" s="34"/>
+      <c r="AB7" s="35"/>
+      <c r="AC7" s="36"/>
+      <c r="AD7" s="34"/>
+      <c r="AE7" s="35"/>
+      <c r="AF7" s="28"/>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" s="16">
@@ -1276,28 +1289,28 @@
       <c r="H8" s="10">
         <v>0.94558600000000004</v>
       </c>
-      <c r="K8" s="44"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="46"/>
-      <c r="N8" s="47"/>
-      <c r="O8" s="47"/>
-      <c r="P8" s="46"/>
-      <c r="Q8" s="47"/>
-      <c r="R8" s="47"/>
-      <c r="S8" s="46"/>
-      <c r="T8" s="47"/>
-      <c r="U8" s="39"/>
-      <c r="V8" s="44"/>
-      <c r="W8" s="50"/>
-      <c r="X8" s="46"/>
-      <c r="Y8" s="47"/>
-      <c r="Z8" s="48"/>
-      <c r="AA8" s="46"/>
-      <c r="AB8" s="47"/>
-      <c r="AC8" s="48"/>
-      <c r="AD8" s="46"/>
-      <c r="AE8" s="47"/>
-      <c r="AF8" s="39"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="37"/>
+      <c r="M8" s="34"/>
+      <c r="N8" s="35"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="34"/>
+      <c r="Q8" s="35"/>
+      <c r="R8" s="35"/>
+      <c r="S8" s="34"/>
+      <c r="T8" s="35"/>
+      <c r="U8" s="28"/>
+      <c r="V8" s="32"/>
+      <c r="W8" s="38"/>
+      <c r="X8" s="34"/>
+      <c r="Y8" s="35"/>
+      <c r="Z8" s="36"/>
+      <c r="AA8" s="34"/>
+      <c r="AB8" s="35"/>
+      <c r="AC8" s="36"/>
+      <c r="AD8" s="34"/>
+      <c r="AE8" s="35"/>
+      <c r="AF8" s="28"/>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A9" s="16">
@@ -1324,28 +1337,28 @@
       <c r="H9" s="10">
         <v>0.94884100000000005</v>
       </c>
-      <c r="K9" s="44"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="46"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="47"/>
-      <c r="P9" s="46"/>
-      <c r="Q9" s="47"/>
-      <c r="R9" s="47"/>
-      <c r="S9" s="46"/>
-      <c r="T9" s="47"/>
-      <c r="U9" s="39"/>
-      <c r="V9" s="44"/>
-      <c r="W9" s="50"/>
-      <c r="X9" s="46"/>
-      <c r="Y9" s="47"/>
-      <c r="Z9" s="48"/>
-      <c r="AA9" s="46"/>
-      <c r="AB9" s="47"/>
-      <c r="AC9" s="48"/>
-      <c r="AD9" s="46"/>
-      <c r="AE9" s="47"/>
-      <c r="AF9" s="39"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="35"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="34"/>
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
+      <c r="S9" s="34"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="28"/>
+      <c r="V9" s="32"/>
+      <c r="W9" s="38"/>
+      <c r="X9" s="34"/>
+      <c r="Y9" s="35"/>
+      <c r="Z9" s="36"/>
+      <c r="AA9" s="34"/>
+      <c r="AB9" s="35"/>
+      <c r="AC9" s="36"/>
+      <c r="AD9" s="34"/>
+      <c r="AE9" s="35"/>
+      <c r="AF9" s="28"/>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A10" s="16">
@@ -1372,28 +1385,28 @@
       <c r="H10" s="10">
         <v>0.95210399999999995</v>
       </c>
-      <c r="K10" s="44"/>
-      <c r="L10" s="49"/>
-      <c r="M10" s="46"/>
-      <c r="N10" s="47"/>
-      <c r="O10" s="47"/>
-      <c r="P10" s="46"/>
-      <c r="Q10" s="47"/>
-      <c r="R10" s="47"/>
-      <c r="S10" s="46"/>
-      <c r="T10" s="47"/>
-      <c r="U10" s="39"/>
-      <c r="V10" s="44"/>
-      <c r="W10" s="50"/>
-      <c r="X10" s="46"/>
-      <c r="Y10" s="47"/>
-      <c r="Z10" s="48"/>
-      <c r="AA10" s="46"/>
-      <c r="AB10" s="47"/>
-      <c r="AC10" s="48"/>
-      <c r="AD10" s="46"/>
-      <c r="AE10" s="47"/>
-      <c r="AF10" s="39"/>
+      <c r="K10" s="32"/>
+      <c r="L10" s="37"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="35"/>
+      <c r="O10" s="35"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="35"/>
+      <c r="R10" s="35"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="35"/>
+      <c r="U10" s="28"/>
+      <c r="V10" s="32"/>
+      <c r="W10" s="38"/>
+      <c r="X10" s="34"/>
+      <c r="Y10" s="35"/>
+      <c r="Z10" s="36"/>
+      <c r="AA10" s="34"/>
+      <c r="AB10" s="35"/>
+      <c r="AC10" s="36"/>
+      <c r="AD10" s="34"/>
+      <c r="AE10" s="35"/>
+      <c r="AF10" s="28"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A11" s="16">
@@ -1420,28 +1433,28 @@
       <c r="H11" s="10">
         <v>0.95527700000000004</v>
       </c>
-      <c r="K11" s="44"/>
-      <c r="L11" s="49"/>
-      <c r="M11" s="46"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="47"/>
-      <c r="P11" s="46"/>
-      <c r="Q11" s="47"/>
-      <c r="R11" s="47"/>
-      <c r="S11" s="46"/>
-      <c r="T11" s="47"/>
-      <c r="U11" s="39"/>
-      <c r="V11" s="44"/>
-      <c r="W11" s="50"/>
-      <c r="X11" s="46"/>
-      <c r="Y11" s="47"/>
-      <c r="Z11" s="48"/>
-      <c r="AA11" s="46"/>
-      <c r="AB11" s="47"/>
-      <c r="AC11" s="48"/>
-      <c r="AD11" s="46"/>
-      <c r="AE11" s="47"/>
-      <c r="AF11" s="39"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="37"/>
+      <c r="M11" s="34"/>
+      <c r="N11" s="35"/>
+      <c r="O11" s="35"/>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="35"/>
+      <c r="R11" s="35"/>
+      <c r="S11" s="34"/>
+      <c r="T11" s="35"/>
+      <c r="U11" s="28"/>
+      <c r="V11" s="32"/>
+      <c r="W11" s="38"/>
+      <c r="X11" s="34"/>
+      <c r="Y11" s="35"/>
+      <c r="Z11" s="36"/>
+      <c r="AA11" s="34"/>
+      <c r="AB11" s="35"/>
+      <c r="AC11" s="36"/>
+      <c r="AD11" s="34"/>
+      <c r="AE11" s="35"/>
+      <c r="AF11" s="28"/>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A12" s="16">
@@ -1468,28 +1481,28 @@
       <c r="H12" s="10">
         <v>0.95825199999999999</v>
       </c>
-      <c r="K12" s="44"/>
-      <c r="L12" s="49"/>
-      <c r="M12" s="46"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="47"/>
-      <c r="P12" s="46"/>
-      <c r="Q12" s="47"/>
-      <c r="R12" s="47"/>
-      <c r="S12" s="46"/>
-      <c r="T12" s="47"/>
-      <c r="U12" s="39"/>
-      <c r="V12" s="44"/>
-      <c r="W12" s="50"/>
-      <c r="X12" s="46"/>
-      <c r="Y12" s="47"/>
-      <c r="Z12" s="48"/>
-      <c r="AA12" s="46"/>
-      <c r="AB12" s="47"/>
-      <c r="AC12" s="48"/>
-      <c r="AD12" s="46"/>
-      <c r="AE12" s="47"/>
-      <c r="AF12" s="39"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="37"/>
+      <c r="M12" s="34"/>
+      <c r="N12" s="35"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="34"/>
+      <c r="Q12" s="35"/>
+      <c r="R12" s="35"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="35"/>
+      <c r="U12" s="28"/>
+      <c r="V12" s="32"/>
+      <c r="W12" s="38"/>
+      <c r="X12" s="34"/>
+      <c r="Y12" s="35"/>
+      <c r="Z12" s="36"/>
+      <c r="AA12" s="34"/>
+      <c r="AB12" s="35"/>
+      <c r="AC12" s="36"/>
+      <c r="AD12" s="34"/>
+      <c r="AE12" s="35"/>
+      <c r="AF12" s="28"/>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A13" s="16">
@@ -1516,28 +1529,28 @@
       <c r="H13" s="10">
         <v>0.96092699999999998</v>
       </c>
-      <c r="K13" s="44"/>
-      <c r="L13" s="49"/>
-      <c r="M13" s="46"/>
-      <c r="N13" s="47"/>
-      <c r="O13" s="47"/>
-      <c r="P13" s="46"/>
-      <c r="Q13" s="47"/>
-      <c r="R13" s="47"/>
-      <c r="S13" s="46"/>
-      <c r="T13" s="47"/>
-      <c r="U13" s="39"/>
-      <c r="V13" s="44"/>
-      <c r="W13" s="50"/>
-      <c r="X13" s="46"/>
-      <c r="Y13" s="47"/>
-      <c r="Z13" s="48"/>
-      <c r="AA13" s="46"/>
-      <c r="AB13" s="47"/>
-      <c r="AC13" s="48"/>
-      <c r="AD13" s="46"/>
-      <c r="AE13" s="47"/>
-      <c r="AF13" s="39"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="37"/>
+      <c r="M13" s="34"/>
+      <c r="N13" s="35"/>
+      <c r="O13" s="35"/>
+      <c r="P13" s="34"/>
+      <c r="Q13" s="35"/>
+      <c r="R13" s="35"/>
+      <c r="S13" s="34"/>
+      <c r="T13" s="35"/>
+      <c r="U13" s="28"/>
+      <c r="V13" s="32"/>
+      <c r="W13" s="38"/>
+      <c r="X13" s="34"/>
+      <c r="Y13" s="35"/>
+      <c r="Z13" s="36"/>
+      <c r="AA13" s="34"/>
+      <c r="AB13" s="35"/>
+      <c r="AC13" s="36"/>
+      <c r="AD13" s="34"/>
+      <c r="AE13" s="35"/>
+      <c r="AF13" s="28"/>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A14" s="16">
@@ -1564,28 +1577,28 @@
       <c r="H14" s="10">
         <v>0.96322399999999997</v>
       </c>
-      <c r="K14" s="44"/>
-      <c r="L14" s="49"/>
-      <c r="M14" s="46"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="47"/>
-      <c r="P14" s="46"/>
-      <c r="Q14" s="47"/>
-      <c r="R14" s="47"/>
-      <c r="S14" s="46"/>
-      <c r="T14" s="47"/>
-      <c r="U14" s="39"/>
-      <c r="V14" s="44"/>
-      <c r="W14" s="50"/>
-      <c r="X14" s="46"/>
-      <c r="Y14" s="47"/>
-      <c r="Z14" s="48"/>
-      <c r="AA14" s="46"/>
-      <c r="AB14" s="47"/>
-      <c r="AC14" s="48"/>
-      <c r="AD14" s="46"/>
-      <c r="AE14" s="47"/>
-      <c r="AF14" s="39"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="37"/>
+      <c r="M14" s="34"/>
+      <c r="N14" s="35"/>
+      <c r="O14" s="35"/>
+      <c r="P14" s="34"/>
+      <c r="Q14" s="35"/>
+      <c r="R14" s="35"/>
+      <c r="S14" s="34"/>
+      <c r="T14" s="35"/>
+      <c r="U14" s="28"/>
+      <c r="V14" s="32"/>
+      <c r="W14" s="38"/>
+      <c r="X14" s="34"/>
+      <c r="Y14" s="35"/>
+      <c r="Z14" s="36"/>
+      <c r="AA14" s="34"/>
+      <c r="AB14" s="35"/>
+      <c r="AC14" s="36"/>
+      <c r="AD14" s="34"/>
+      <c r="AE14" s="35"/>
+      <c r="AF14" s="28"/>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A15" s="17">
@@ -1612,52 +1625,56 @@
       <c r="H15" s="11">
         <v>0.96509999999999996</v>
       </c>
-      <c r="K15" s="44"/>
-      <c r="L15" s="49"/>
-      <c r="M15" s="46"/>
-      <c r="N15" s="47"/>
-      <c r="O15" s="47"/>
-      <c r="P15" s="46"/>
-      <c r="Q15" s="47"/>
-      <c r="R15" s="47"/>
-      <c r="S15" s="46"/>
-      <c r="T15" s="47"/>
-      <c r="U15" s="39"/>
-      <c r="V15" s="44"/>
-      <c r="W15" s="50"/>
-      <c r="X15" s="46"/>
-      <c r="Y15" s="47"/>
-      <c r="Z15" s="48"/>
-      <c r="AA15" s="46"/>
-      <c r="AB15" s="47"/>
-      <c r="AC15" s="48"/>
-      <c r="AD15" s="46"/>
-      <c r="AE15" s="47"/>
-      <c r="AF15" s="39"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="37"/>
+      <c r="M15" s="34"/>
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="34"/>
+      <c r="Q15" s="35"/>
+      <c r="R15" s="35"/>
+      <c r="S15" s="34"/>
+      <c r="T15" s="35"/>
+      <c r="U15" s="28"/>
+      <c r="V15" s="32"/>
+      <c r="W15" s="38"/>
+      <c r="X15" s="34"/>
+      <c r="Y15" s="35"/>
+      <c r="Z15" s="36"/>
+      <c r="AA15" s="34"/>
+      <c r="AB15" s="35"/>
+      <c r="AC15" s="36"/>
+      <c r="AD15" s="34"/>
+      <c r="AE15" s="35"/>
+      <c r="AF15" s="28"/>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
-      <c r="O16" s="39"/>
-      <c r="P16" s="39"/>
-      <c r="Q16" s="39"/>
-      <c r="R16" s="39"/>
-      <c r="S16" s="39"/>
-      <c r="T16" s="39"/>
-      <c r="U16" s="39"/>
-      <c r="V16" s="39"/>
-      <c r="W16" s="39"/>
-      <c r="X16" s="39"/>
-      <c r="Y16" s="39"/>
-      <c r="Z16" s="39"/>
-      <c r="AA16" s="39"/>
-      <c r="AB16" s="39"/>
-      <c r="AC16" s="39"/>
-      <c r="AD16" s="39"/>
-      <c r="AE16" s="39"/>
-      <c r="AF16" s="39"/>
+      <c r="K16" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="L16" s="28"/>
+      <c r="M16" s="28"/>
+      <c r="N16" s="28"/>
+      <c r="O16" s="28"/>
+      <c r="P16" s="28"/>
+      <c r="Q16" s="28"/>
+      <c r="R16" s="28"/>
+      <c r="S16" s="28"/>
+      <c r="T16" s="28"/>
+      <c r="U16" s="28"/>
+      <c r="V16" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="W16" s="28"/>
+      <c r="X16" s="28"/>
+      <c r="Y16" s="28"/>
+      <c r="Z16" s="28"/>
+      <c r="AA16" s="28"/>
+      <c r="AB16" s="28"/>
+      <c r="AC16" s="28"/>
+      <c r="AD16" s="28"/>
+      <c r="AE16" s="28"/>
+      <c r="AF16" s="28"/>
     </row>
     <row r="17" spans="11:31" x14ac:dyDescent="0.3">
       <c r="K17" t="s">
@@ -1681,37 +1698,37 @@
     </row>
     <row r="18" spans="11:31" x14ac:dyDescent="0.3">
       <c r="K18" s="13"/>
-      <c r="L18" s="31" t="s">
+      <c r="L18" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="M18" s="31"/>
-      <c r="N18" s="31"/>
-      <c r="O18" s="31" t="s">
+      <c r="M18" s="41"/>
+      <c r="N18" s="41"/>
+      <c r="O18" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="P18" s="31"/>
-      <c r="Q18" s="23"/>
-      <c r="R18" s="23" t="s">
+      <c r="P18" s="41"/>
+      <c r="Q18" s="39"/>
+      <c r="R18" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="S18" s="23"/>
-      <c r="T18" s="38"/>
+      <c r="S18" s="39"/>
+      <c r="T18" s="40"/>
       <c r="V18" s="13"/>
-      <c r="W18" s="31" t="s">
+      <c r="W18" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="X18" s="31"/>
-      <c r="Y18" s="31"/>
-      <c r="Z18" s="31" t="s">
+      <c r="X18" s="41"/>
+      <c r="Y18" s="41"/>
+      <c r="Z18" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="AA18" s="31"/>
-      <c r="AB18" s="31"/>
-      <c r="AC18" s="23" t="s">
+      <c r="AA18" s="41"/>
+      <c r="AB18" s="41"/>
+      <c r="AC18" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="AD18" s="23"/>
-      <c r="AE18" s="38"/>
+      <c r="AD18" s="39"/>
+      <c r="AE18" s="40"/>
     </row>
     <row r="19" spans="11:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="K19" s="14" t="s">
@@ -1813,12 +1830,12 @@
         <v>155.1</v>
       </c>
       <c r="X20" s="19">
-        <v>1.9836</v>
+        <v>1.9836800000000001</v>
       </c>
       <c r="Y20" s="9">
-        <v>0.73329999999999995</v>
-      </c>
-      <c r="Z20" s="35">
+        <v>0.733317</v>
+      </c>
+      <c r="Z20" s="25">
         <v>155.1</v>
       </c>
       <c r="AA20" s="19">
@@ -1827,7 +1844,7 @@
       <c r="AB20" s="9">
         <v>0.87204000000000004</v>
       </c>
-      <c r="AC20" s="35">
+      <c r="AC20" s="25">
         <v>155.1</v>
       </c>
       <c r="AD20" s="19">
@@ -1875,28 +1892,28 @@
         <v>186.7</v>
       </c>
       <c r="X21" s="20">
-        <v>1.9866999999999999</v>
+        <v>1.9867900000000001</v>
       </c>
       <c r="Y21" s="10">
-        <v>0.73440000000000005</v>
-      </c>
-      <c r="Z21" s="36">
+        <v>0.73446599999999995</v>
+      </c>
+      <c r="Z21" s="26">
         <v>186.7</v>
       </c>
       <c r="AA21" s="20">
         <v>4.8747299999999996</v>
       </c>
       <c r="AB21" s="10">
-        <v>0.87466999999999995</v>
-      </c>
-      <c r="AC21" s="36">
+        <v>0.87467200000000001</v>
+      </c>
+      <c r="AC21" s="26">
         <v>186.7</v>
       </c>
       <c r="AD21" s="20">
         <v>13.129300000000001</v>
       </c>
       <c r="AE21" s="10">
-        <v>0.93601999999999996</v>
+        <v>0.93602700000000005</v>
       </c>
     </row>
     <row r="22" spans="11:31" x14ac:dyDescent="0.3">
@@ -1933,17 +1950,17 @@
       <c r="V22" s="16">
         <v>2027</v>
       </c>
-      <c r="W22" s="33">
+      <c r="W22" s="23">
         <v>881.5</v>
       </c>
       <c r="X22" s="20">
-        <v>1.9873000000000001</v>
+        <v>1.98732</v>
       </c>
       <c r="Y22" s="10">
-        <v>0.73460000000000003</v>
-      </c>
-      <c r="Z22" s="36">
-        <v>881.5</v>
+        <v>0.73465999999999998</v>
+      </c>
+      <c r="Z22" s="26">
+        <v>843.85199999999998</v>
       </c>
       <c r="AA22" s="20">
         <v>4.8882700000000003</v>
@@ -1951,7 +1968,7 @@
       <c r="AB22" s="10">
         <v>0.87709999999999999</v>
       </c>
-      <c r="AC22" s="36">
+      <c r="AC22" s="26">
         <v>881.5</v>
       </c>
       <c r="AD22" s="20">
@@ -1995,32 +2012,32 @@
       <c r="V23" s="16">
         <v>2028</v>
       </c>
-      <c r="W23" s="33">
+      <c r="W23" s="23">
         <v>865.88</v>
       </c>
       <c r="X23" s="20">
-        <v>1.9038999999999999</v>
+        <v>1.90828</v>
       </c>
       <c r="Y23" s="10">
-        <v>0.70379999999999998</v>
-      </c>
-      <c r="Z23" s="36">
+        <v>0.70544200000000001</v>
+      </c>
+      <c r="Z23" s="26">
+        <v>825.65499999999997</v>
+      </c>
+      <c r="AA23" s="20">
+        <v>4.8214499999999996</v>
+      </c>
+      <c r="AB23" s="10">
+        <v>0.86511000000000005</v>
+      </c>
+      <c r="AC23" s="26">
         <v>865.88</v>
       </c>
-      <c r="AA23" s="20">
-        <v>4.8167499999999999</v>
-      </c>
-      <c r="AB23" s="10">
-        <v>0.86426000000000003</v>
-      </c>
-      <c r="AC23" s="36">
-        <v>865.88</v>
-      </c>
       <c r="AD23" s="20">
-        <v>13.1439</v>
+        <v>13.148300000000001</v>
       </c>
       <c r="AE23" s="10">
-        <v>0.93706</v>
+        <v>0.93738200000000005</v>
       </c>
     </row>
     <row r="24" spans="11:31" x14ac:dyDescent="0.3">
@@ -2057,32 +2074,32 @@
       <c r="V24" s="16">
         <v>2029</v>
       </c>
-      <c r="W24" s="33">
+      <c r="W24" s="23">
         <v>849.55</v>
       </c>
       <c r="X24" s="20">
-        <v>1.8230999999999999</v>
+        <v>1.8321499999999999</v>
       </c>
       <c r="Y24" s="10">
-        <v>0.67390000000000005</v>
-      </c>
-      <c r="Z24" s="36">
+        <v>0.67729899999999998</v>
+      </c>
+      <c r="Z24" s="26">
+        <v>808.75199999999995</v>
+      </c>
+      <c r="AA24" s="20">
+        <v>4.7584</v>
+      </c>
+      <c r="AB24" s="10">
+        <v>0.85379799999999995</v>
+      </c>
+      <c r="AC24" s="26">
         <v>849.55</v>
       </c>
-      <c r="AA24" s="20">
-        <v>4.74871</v>
-      </c>
-      <c r="AB24" s="10">
-        <v>0.85204999999999997</v>
-      </c>
-      <c r="AC24" s="36">
-        <v>849.55</v>
-      </c>
       <c r="AD24" s="20">
-        <v>13.115399999999999</v>
+        <v>13.124599999999999</v>
       </c>
       <c r="AE24" s="10">
-        <v>0.93503000000000003</v>
+        <v>0.93569199999999997</v>
       </c>
     </row>
     <row r="25" spans="11:31" x14ac:dyDescent="0.3">
@@ -2119,32 +2136,32 @@
       <c r="V25" s="16">
         <v>2030</v>
       </c>
-      <c r="W25" s="33">
+      <c r="W25" s="23">
         <v>833.53</v>
       </c>
       <c r="X25" s="20">
-        <v>1.7445999999999999</v>
+        <v>1.75857</v>
       </c>
       <c r="Y25" s="10">
-        <v>0.64490000000000003</v>
-      </c>
-      <c r="Z25" s="36">
+        <v>0.65009700000000004</v>
+      </c>
+      <c r="Z25" s="26">
+        <v>792.19500000000005</v>
+      </c>
+      <c r="AA25" s="20">
+        <v>4.6984399999999997</v>
+      </c>
+      <c r="AB25" s="10">
+        <v>0.84303899999999998</v>
+      </c>
+      <c r="AC25" s="26">
         <v>833.53</v>
       </c>
-      <c r="AA25" s="20">
-        <v>4.6837099999999996</v>
-      </c>
-      <c r="AB25" s="10">
-        <v>0.84038999999999997</v>
-      </c>
-      <c r="AC25" s="36">
-        <v>833.53</v>
-      </c>
       <c r="AD25" s="20">
-        <v>13.0907</v>
+        <v>13.104799999999999</v>
       </c>
       <c r="AE25" s="10">
-        <v>0.93327000000000004</v>
+        <v>0.93428299999999997</v>
       </c>
     </row>
     <row r="26" spans="11:31" x14ac:dyDescent="0.3">
@@ -2181,32 +2198,32 @@
       <c r="V26" s="16">
         <v>2031</v>
       </c>
-      <c r="W26" s="33">
+      <c r="W26" s="23">
         <v>817.84</v>
       </c>
       <c r="X26" s="20">
-        <v>1.6685000000000001</v>
+        <v>1.6874100000000001</v>
       </c>
       <c r="Y26" s="10">
-        <v>0.61680000000000001</v>
-      </c>
-      <c r="Z26" s="36">
+        <v>0.62379399999999996</v>
+      </c>
+      <c r="Z26" s="26">
+        <v>775.98299999999995</v>
+      </c>
+      <c r="AA26" s="20">
+        <v>4.6411300000000004</v>
+      </c>
+      <c r="AB26" s="10">
+        <v>0.83275600000000005</v>
+      </c>
+      <c r="AC26" s="26">
         <v>817.84</v>
       </c>
-      <c r="AA26" s="20">
-        <v>4.6213499999999996</v>
-      </c>
-      <c r="AB26" s="10">
-        <v>0.82920000000000005</v>
-      </c>
-      <c r="AC26" s="36">
-        <v>817.84</v>
-      </c>
       <c r="AD26" s="20">
-        <v>13.0686</v>
+        <v>13.0878</v>
       </c>
       <c r="AE26" s="10">
-        <v>0.93169999999999997</v>
+        <v>0.93306900000000004</v>
       </c>
     </row>
     <row r="27" spans="11:31" x14ac:dyDescent="0.3">
@@ -2243,32 +2260,32 @@
       <c r="V27" s="16">
         <v>2032</v>
       </c>
-      <c r="W27" s="33">
+      <c r="W27" s="23">
         <v>803.31</v>
       </c>
       <c r="X27" s="20">
-        <v>1.5945</v>
+        <v>1.6185799999999999</v>
       </c>
       <c r="Y27" s="10">
-        <v>0.58940000000000003</v>
-      </c>
-      <c r="Z27" s="36">
+        <v>0.59834900000000002</v>
+      </c>
+      <c r="Z27" s="26">
+        <v>760.04200000000003</v>
+      </c>
+      <c r="AA27" s="20">
+        <v>4.5860300000000001</v>
+      </c>
+      <c r="AB27" s="10">
+        <v>0.82286999999999999</v>
+      </c>
+      <c r="AC27" s="26">
         <v>803.31</v>
       </c>
-      <c r="AA27" s="20">
-        <v>4.5611800000000002</v>
-      </c>
-      <c r="AB27" s="10">
-        <v>0.81840999999999997</v>
-      </c>
-      <c r="AC27" s="36">
-        <v>803.31</v>
-      </c>
       <c r="AD27" s="20">
-        <v>13.0479</v>
+        <v>13.0722</v>
       </c>
       <c r="AE27" s="10">
-        <v>0.93022000000000005</v>
+        <v>0.93195700000000004</v>
       </c>
     </row>
     <row r="28" spans="11:31" x14ac:dyDescent="0.3">
@@ -2305,32 +2322,32 @@
       <c r="V28" s="16">
         <v>2033</v>
       </c>
-      <c r="W28" s="33">
+      <c r="W28" s="23">
         <v>787.99</v>
       </c>
       <c r="X28" s="20">
-        <v>1.5226</v>
+        <v>1.55193</v>
       </c>
       <c r="Y28" s="10">
-        <v>0.56279999999999997</v>
-      </c>
-      <c r="Z28" s="36">
+        <v>0.57371099999999997</v>
+      </c>
+      <c r="Z28" s="26">
+        <v>745.17600000000004</v>
+      </c>
+      <c r="AA28" s="20">
+        <v>4.5326500000000003</v>
+      </c>
+      <c r="AB28" s="10">
+        <v>0.81329200000000001</v>
+      </c>
+      <c r="AC28" s="26">
         <v>787.99</v>
       </c>
-      <c r="AA28" s="20">
-        <v>4.5026099999999998</v>
-      </c>
-      <c r="AB28" s="10">
-        <v>0.80789999999999995</v>
-      </c>
-      <c r="AC28" s="36">
-        <v>787.99</v>
-      </c>
       <c r="AD28" s="20">
-        <v>13.026899999999999</v>
+        <v>13.0566</v>
       </c>
       <c r="AE28" s="10">
-        <v>0.92871999999999999</v>
+        <v>0.93084199999999995</v>
       </c>
     </row>
     <row r="29" spans="11:31" x14ac:dyDescent="0.3">
@@ -2367,32 +2384,32 @@
       <c r="V29" s="16">
         <v>2034</v>
       </c>
-      <c r="W29" s="33">
+      <c r="W29" s="23">
         <v>773.63</v>
       </c>
       <c r="X29" s="20">
-        <v>1.4525999999999999</v>
+        <v>1.4872099999999999</v>
       </c>
       <c r="Y29" s="10">
-        <v>0.53690000000000004</v>
-      </c>
-      <c r="Z29" s="36">
+        <v>0.54978400000000005</v>
+      </c>
+      <c r="Z29" s="26">
+        <v>729.48900000000003</v>
+      </c>
+      <c r="AA29" s="20">
+        <v>4.48041</v>
+      </c>
+      <c r="AB29" s="10">
+        <v>0.80391800000000002</v>
+      </c>
+      <c r="AC29" s="26">
         <v>773.63</v>
       </c>
-      <c r="AA29" s="20">
-        <v>4.4452999999999996</v>
-      </c>
-      <c r="AB29" s="10">
-        <v>0.79761000000000004</v>
-      </c>
-      <c r="AC29" s="36">
-        <v>773.63</v>
-      </c>
       <c r="AD29" s="20">
-        <v>13.0044</v>
+        <v>13.039400000000001</v>
       </c>
       <c r="AE29" s="10">
-        <v>0.92712000000000006</v>
+        <v>0.92962</v>
       </c>
     </row>
     <row r="30" spans="11:31" x14ac:dyDescent="0.3">
@@ -2429,32 +2446,32 @@
       <c r="V30" s="16">
         <v>2035</v>
       </c>
-      <c r="W30" s="33">
+      <c r="W30" s="23">
         <v>758.44</v>
       </c>
       <c r="X30" s="20">
-        <v>1.3843000000000001</v>
+        <v>1.42441</v>
       </c>
       <c r="Y30" s="10">
-        <v>0.51170000000000004</v>
-      </c>
-      <c r="Z30" s="36">
+        <v>0.52656899999999995</v>
+      </c>
+      <c r="Z30" s="26">
+        <v>713.91499999999996</v>
+      </c>
+      <c r="AA30" s="20">
+        <v>4.4290799999999999</v>
+      </c>
+      <c r="AB30" s="10">
+        <v>0.79470700000000005</v>
+      </c>
+      <c r="AC30" s="26">
         <v>758.44</v>
       </c>
-      <c r="AA30" s="20">
-        <v>4.3887999999999998</v>
-      </c>
-      <c r="AB30" s="10">
-        <v>0.78747999999999996</v>
-      </c>
-      <c r="AC30" s="36">
-        <v>758.44</v>
-      </c>
       <c r="AD30" s="20">
-        <v>12.9794</v>
+        <v>13.0198</v>
       </c>
       <c r="AE30" s="10">
-        <v>0.92534000000000005</v>
+        <v>0.92822300000000002</v>
       </c>
     </row>
     <row r="31" spans="11:31" x14ac:dyDescent="0.3">
@@ -2491,42 +2508,36 @@
       <c r="V31" s="17">
         <v>2036</v>
       </c>
-      <c r="W31" s="34">
+      <c r="W31" s="24">
         <v>744.28</v>
       </c>
       <c r="X31" s="22">
-        <v>1.3180000000000001</v>
+        <v>1.36351</v>
       </c>
       <c r="Y31" s="11">
-        <v>0.48720000000000002</v>
-      </c>
-      <c r="Z31" s="37">
+        <v>0.50405599999999995</v>
+      </c>
+      <c r="Z31" s="27">
+        <v>699.38699999999994</v>
+      </c>
+      <c r="AA31" s="21">
+        <v>4.3784999999999998</v>
+      </c>
+      <c r="AB31" s="11">
+        <v>0.78563300000000003</v>
+      </c>
+      <c r="AC31" s="27">
         <v>744.28</v>
       </c>
-      <c r="AA31" s="21">
-        <v>4.3330799999999998</v>
-      </c>
-      <c r="AB31" s="11">
-        <v>0.77747999999999995</v>
-      </c>
-      <c r="AC31" s="37">
-        <v>744.28</v>
-      </c>
       <c r="AD31" s="21">
-        <v>12.9514</v>
+        <v>12.997299999999999</v>
       </c>
       <c r="AE31" s="11">
-        <v>0.92334000000000005</v>
+        <v>0.92661400000000005</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="AC18:AE18"/>
-    <mergeCell ref="L18:N18"/>
-    <mergeCell ref="O18:Q18"/>
-    <mergeCell ref="R18:T18"/>
-    <mergeCell ref="W18:Y18"/>
-    <mergeCell ref="Z18:AB18"/>
     <mergeCell ref="W2:Y2"/>
     <mergeCell ref="Z2:AB2"/>
     <mergeCell ref="AC2:AE2"/>
@@ -2537,6 +2548,12 @@
     <mergeCell ref="L2:N2"/>
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="R2:T2"/>
+    <mergeCell ref="AC18:AE18"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="R18:T18"/>
+    <mergeCell ref="W18:Y18"/>
+    <mergeCell ref="Z18:AB18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3234,7 +3251,7 @@
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20">
-        <f>B14+1</f>
+        <f t="shared" ref="B20:B51" si="4">B14+1</f>
         <v>2028</v>
       </c>
       <c r="C20">
@@ -3249,7 +3266,7 @@
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21">
-        <f>B15+1</f>
+        <f t="shared" si="4"/>
         <v>2028</v>
       </c>
       <c r="C21">
@@ -3264,7 +3281,7 @@
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22">
-        <f>B16+1</f>
+        <f t="shared" si="4"/>
         <v>2028</v>
       </c>
       <c r="C22">
@@ -3279,7 +3296,7 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23">
-        <f>B17+1</f>
+        <f t="shared" si="4"/>
         <v>2028</v>
       </c>
       <c r="C23">
@@ -3294,7 +3311,7 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24">
-        <f>B18+1</f>
+        <f t="shared" si="4"/>
         <v>2028</v>
       </c>
       <c r="C24">
@@ -3309,7 +3326,7 @@
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25">
-        <f>B19+1</f>
+        <f t="shared" si="4"/>
         <v>2028</v>
       </c>
       <c r="C25">
@@ -3324,7 +3341,7 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26">
-        <f>B20+1</f>
+        <f t="shared" si="4"/>
         <v>2029</v>
       </c>
       <c r="C26">
@@ -3339,7 +3356,7 @@
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27">
-        <f>B21+1</f>
+        <f t="shared" si="4"/>
         <v>2029</v>
       </c>
       <c r="C27">
@@ -3354,7 +3371,7 @@
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28">
-        <f>B22+1</f>
+        <f t="shared" si="4"/>
         <v>2029</v>
       </c>
       <c r="C28">
@@ -3369,7 +3386,7 @@
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29">
-        <f>B23+1</f>
+        <f t="shared" si="4"/>
         <v>2029</v>
       </c>
       <c r="C29">
@@ -3384,7 +3401,7 @@
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30">
-        <f>B24+1</f>
+        <f t="shared" si="4"/>
         <v>2029</v>
       </c>
       <c r="C30">
@@ -3399,7 +3416,7 @@
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31">
-        <f>B25+1</f>
+        <f t="shared" si="4"/>
         <v>2029</v>
       </c>
       <c r="C31">
@@ -3414,7 +3431,7 @@
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32">
-        <f>B26+1</f>
+        <f t="shared" si="4"/>
         <v>2030</v>
       </c>
       <c r="C32">
@@ -3429,7 +3446,7 @@
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33">
-        <f>B27+1</f>
+        <f t="shared" si="4"/>
         <v>2030</v>
       </c>
       <c r="C33">
@@ -3444,7 +3461,7 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34">
-        <f>B28+1</f>
+        <f t="shared" si="4"/>
         <v>2030</v>
       </c>
       <c r="C34">
@@ -3459,7 +3476,7 @@
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35">
-        <f>B29+1</f>
+        <f t="shared" si="4"/>
         <v>2030</v>
       </c>
       <c r="C35">
@@ -3474,7 +3491,7 @@
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36">
-        <f>B30+1</f>
+        <f t="shared" si="4"/>
         <v>2030</v>
       </c>
       <c r="C36">
@@ -3489,7 +3506,7 @@
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B37">
-        <f>B31+1</f>
+        <f t="shared" si="4"/>
         <v>2030</v>
       </c>
       <c r="C37">
@@ -3504,7 +3521,7 @@
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B38">
-        <f>B32+1</f>
+        <f t="shared" si="4"/>
         <v>2031</v>
       </c>
       <c r="C38">
@@ -3519,7 +3536,7 @@
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B39">
-        <f>B33+1</f>
+        <f t="shared" si="4"/>
         <v>2031</v>
       </c>
       <c r="C39">
@@ -3534,7 +3551,7 @@
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B40">
-        <f>B34+1</f>
+        <f t="shared" si="4"/>
         <v>2031</v>
       </c>
       <c r="C40">
@@ -3549,7 +3566,7 @@
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B41">
-        <f>B35+1</f>
+        <f t="shared" si="4"/>
         <v>2031</v>
       </c>
       <c r="C41">
@@ -3564,7 +3581,7 @@
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B42">
-        <f>B36+1</f>
+        <f t="shared" si="4"/>
         <v>2031</v>
       </c>
       <c r="C42">
@@ -3579,7 +3596,7 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B43">
-        <f>B37+1</f>
+        <f t="shared" si="4"/>
         <v>2031</v>
       </c>
       <c r="C43">
@@ -3594,7 +3611,7 @@
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B44">
-        <f>B38+1</f>
+        <f t="shared" si="4"/>
         <v>2032</v>
       </c>
       <c r="C44">
@@ -3609,7 +3626,7 @@
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B45">
-        <f>B39+1</f>
+        <f t="shared" si="4"/>
         <v>2032</v>
       </c>
       <c r="C45">
@@ -3624,7 +3641,7 @@
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B46">
-        <f>B40+1</f>
+        <f t="shared" si="4"/>
         <v>2032</v>
       </c>
       <c r="C46">
@@ -3639,7 +3656,7 @@
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B47">
-        <f>B41+1</f>
+        <f t="shared" si="4"/>
         <v>2032</v>
       </c>
       <c r="C47">
@@ -3654,7 +3671,7 @@
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B48">
-        <f>B42+1</f>
+        <f t="shared" si="4"/>
         <v>2032</v>
       </c>
       <c r="C48">
@@ -3669,7 +3686,7 @@
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B49">
-        <f>B43+1</f>
+        <f t="shared" si="4"/>
         <v>2032</v>
       </c>
       <c r="C49">
@@ -3684,7 +3701,7 @@
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B50">
-        <f>B44+1</f>
+        <f t="shared" si="4"/>
         <v>2033</v>
       </c>
       <c r="C50">
@@ -3699,7 +3716,7 @@
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B51">
-        <f>B45+1</f>
+        <f t="shared" si="4"/>
         <v>2033</v>
       </c>
       <c r="C51">
@@ -3714,7 +3731,7 @@
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B52">
-        <f>B46+1</f>
+        <f t="shared" ref="B52:B83" si="5">B46+1</f>
         <v>2033</v>
       </c>
       <c r="C52">
@@ -3729,7 +3746,7 @@
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B53">
-        <f>B47+1</f>
+        <f t="shared" si="5"/>
         <v>2033</v>
       </c>
       <c r="C53">
@@ -3744,7 +3761,7 @@
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B54">
-        <f>B48+1</f>
+        <f t="shared" si="5"/>
         <v>2033</v>
       </c>
       <c r="C54">
@@ -3759,7 +3776,7 @@
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B55">
-        <f>B49+1</f>
+        <f t="shared" si="5"/>
         <v>2033</v>
       </c>
       <c r="C55">
@@ -3774,7 +3791,7 @@
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B56">
-        <f>B50+1</f>
+        <f t="shared" si="5"/>
         <v>2034</v>
       </c>
       <c r="C56">
@@ -3789,7 +3806,7 @@
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B57">
-        <f>B51+1</f>
+        <f t="shared" si="5"/>
         <v>2034</v>
       </c>
       <c r="C57">
@@ -3804,7 +3821,7 @@
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B58">
-        <f>B52+1</f>
+        <f t="shared" si="5"/>
         <v>2034</v>
       </c>
       <c r="C58">
@@ -3819,7 +3836,7 @@
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B59">
-        <f>B53+1</f>
+        <f t="shared" si="5"/>
         <v>2034</v>
       </c>
       <c r="C59">
@@ -3834,7 +3851,7 @@
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B60">
-        <f>B54+1</f>
+        <f t="shared" si="5"/>
         <v>2034</v>
       </c>
       <c r="C60">
@@ -3849,7 +3866,7 @@
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B61">
-        <f>B55+1</f>
+        <f t="shared" si="5"/>
         <v>2034</v>
       </c>
       <c r="C61">
@@ -3864,7 +3881,7 @@
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B62">
-        <f>B56+1</f>
+        <f t="shared" si="5"/>
         <v>2035</v>
       </c>
       <c r="C62">
@@ -3879,7 +3896,7 @@
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B63">
-        <f>B57+1</f>
+        <f t="shared" si="5"/>
         <v>2035</v>
       </c>
       <c r="C63">
@@ -3894,7 +3911,7 @@
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B64">
-        <f>B58+1</f>
+        <f t="shared" si="5"/>
         <v>2035</v>
       </c>
       <c r="C64">
@@ -3909,7 +3926,7 @@
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B65">
-        <f>B59+1</f>
+        <f t="shared" si="5"/>
         <v>2035</v>
       </c>
       <c r="C65">
@@ -3924,7 +3941,7 @@
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B66">
-        <f>B60+1</f>
+        <f t="shared" si="5"/>
         <v>2035</v>
       </c>
       <c r="C66">
@@ -3939,7 +3956,7 @@
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B67">
-        <f>B61+1</f>
+        <f t="shared" si="5"/>
         <v>2035</v>
       </c>
       <c r="C67">
@@ -3954,7 +3971,7 @@
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B68">
-        <f>B62+1</f>
+        <f t="shared" si="5"/>
         <v>2036</v>
       </c>
       <c r="C68">
@@ -3969,7 +3986,7 @@
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B69">
-        <f>B63+1</f>
+        <f t="shared" si="5"/>
         <v>2036</v>
       </c>
       <c r="C69">
@@ -3984,7 +4001,7 @@
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B70">
-        <f>B64+1</f>
+        <f t="shared" si="5"/>
         <v>2036</v>
       </c>
       <c r="C70">
@@ -3999,7 +4016,7 @@
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B71">
-        <f>B65+1</f>
+        <f t="shared" si="5"/>
         <v>2036</v>
       </c>
       <c r="C71">
@@ -4014,7 +4031,7 @@
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B72">
-        <f>B66+1</f>
+        <f t="shared" si="5"/>
         <v>2036</v>
       </c>
       <c r="C72">
@@ -4029,7 +4046,7 @@
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B73">
-        <f>B67+1</f>
+        <f t="shared" si="5"/>
         <v>2036</v>
       </c>
       <c r="C73">
@@ -4052,4 +4069,1387 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7534C987-B699-46C5-BBCE-D06BA571F11D}">
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>2025</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>1</v>
+      </c>
+      <c r="D1">
+        <v>33</v>
+      </c>
+      <c r="E1">
+        <f>D1/SUM($D$3:$D$8)</f>
+        <v>0.21276595744680851</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>0.1</v>
+      </c>
+      <c r="E2">
+        <f t="shared" ref="E2:E6" si="0">D2/SUM($D$3:$D$8)</f>
+        <v>6.4474532559638954E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>51.8</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="0"/>
+        <v>0.3339780786589297</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2025</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>3.1</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>1.9987105093488073E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2025</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>24.2</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>0.15602836879432624</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>42.9</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.27659574468085107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2026</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7">
+        <f>D7/SUM($D$9:$D$14)</f>
+        <v>0.21484375</v>
+      </c>
+      <c r="F7">
+        <f>SUM(D7:D12)</f>
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2026</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>0.1</v>
+      </c>
+      <c r="E8">
+        <f t="shared" ref="E8:E12" si="1">D8/SUM($D$9:$D$14)</f>
+        <v>6.5104166666666674E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2026</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>51.8</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>0.33723958333333331</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2026</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>3.1</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>2.0182291666666668E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>2026</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>24.2</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>0.15755208333333334</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2026</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>6</v>
+      </c>
+      <c r="D12">
+        <v>74.5</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>0.48502604166666669</v>
+      </c>
+      <c r="G12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2027</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <f>E13*$F$15</f>
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F13">
+        <v>843.85199999999998</v>
+      </c>
+      <c r="G13">
+        <f>SUM(D13:D18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2027</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <f t="shared" ref="D14:D18" si="2">E14*$F$15</f>
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2027</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2027</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2027</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2027</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2028</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <f>E19*$F$21</f>
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F19">
+        <v>825.65499999999997</v>
+      </c>
+      <c r="G19">
+        <f>SUM(D19:D24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2028</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20">
+        <f t="shared" ref="D20:D24" si="3">E20*$F$21</f>
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2028</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>3</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2028</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2028</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2028</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>6</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2029</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <f>E25*$F$27</f>
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F25">
+        <v>808.75199999999995</v>
+      </c>
+      <c r="G25">
+        <f>SUM(D25:D30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2029</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>2</v>
+      </c>
+      <c r="D26">
+        <f t="shared" ref="D26:D30" si="4">E26*$F$27</f>
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2029</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>3</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2029</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>2029</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>2029</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>6</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>2030</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <f>E31*$F$33</f>
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F31">
+        <v>792.19500000000005</v>
+      </c>
+      <c r="G31">
+        <f>SUM(D31:D36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>2030</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32">
+        <v>2</v>
+      </c>
+      <c r="D32">
+        <f t="shared" ref="D32:D36" si="5">E32*$F$33</f>
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>2030</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>3</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>2030</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>2030</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35">
+        <v>5</v>
+      </c>
+      <c r="D35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>2030</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36">
+        <v>6</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>2031</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <f>E37*$F$39</f>
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F37">
+        <v>775.98299999999995</v>
+      </c>
+      <c r="G37">
+        <f>SUM(D37:D42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>2031</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38">
+        <f t="shared" ref="D38:D42" si="6">E38*$F$39</f>
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>2031</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>3</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>2031</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40">
+        <v>4</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>2031</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41">
+        <v>5</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>2031</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42">
+        <v>6</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>2032</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43">
+        <f>E43*$F$45</f>
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F43">
+        <v>760.04200000000003</v>
+      </c>
+      <c r="G43">
+        <f>SUM(D43:D48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>2032</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44">
+        <v>2</v>
+      </c>
+      <c r="D44">
+        <f t="shared" ref="D44:D48" si="7">E44*$F$45</f>
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>2032</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45">
+        <v>3</v>
+      </c>
+      <c r="D45">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>2032</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46">
+        <v>4</v>
+      </c>
+      <c r="D46">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>2032</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47">
+        <v>5</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>2032</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48">
+        <v>6</v>
+      </c>
+      <c r="D48">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>2033</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+      <c r="D49">
+        <f>E49*$F$51</f>
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F49">
+        <v>745.17600000000004</v>
+      </c>
+      <c r="G49">
+        <f>SUM(D49:D54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>2033</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50">
+        <f t="shared" ref="D50:D54" si="8">E50*$F$51</f>
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>2033</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>2033</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52">
+        <v>4</v>
+      </c>
+      <c r="D52">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>2033</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53">
+        <v>5</v>
+      </c>
+      <c r="D53">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>2033</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54">
+        <v>6</v>
+      </c>
+      <c r="D54">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>2034</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55">
+        <v>1</v>
+      </c>
+      <c r="D55">
+        <f>E55*$F$57</f>
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F55">
+        <v>729.48900000000003</v>
+      </c>
+      <c r="G55">
+        <f>SUM(D55:D60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>2034</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56">
+        <v>2</v>
+      </c>
+      <c r="D56">
+        <f t="shared" ref="D56:D60" si="9">E56*$F$57</f>
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>2034</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57">
+        <v>3</v>
+      </c>
+      <c r="D57">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>2034</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58">
+        <v>4</v>
+      </c>
+      <c r="D58">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>2034</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59">
+        <v>5</v>
+      </c>
+      <c r="D59">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>2034</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60">
+        <v>6</v>
+      </c>
+      <c r="D60">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>2035</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+      <c r="D61">
+        <f>E61*$F$63</f>
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F61">
+        <v>713.91499999999996</v>
+      </c>
+      <c r="G61">
+        <f>SUM(D61:D66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>2035</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62">
+        <v>2</v>
+      </c>
+      <c r="D62">
+        <f t="shared" ref="D62:D66" si="10">E62*$F$63</f>
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>2035</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63">
+        <v>3</v>
+      </c>
+      <c r="D63">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>2035</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64">
+        <v>4</v>
+      </c>
+      <c r="D64">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>2035</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65">
+        <v>5</v>
+      </c>
+      <c r="D65">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>2035</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66">
+        <v>6</v>
+      </c>
+      <c r="D66">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>2036</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67">
+        <v>1</v>
+      </c>
+      <c r="D67">
+        <f>E67*$F$69</f>
+        <v>0</v>
+      </c>
+      <c r="E67">
+        <v>0.17675415104445635</v>
+      </c>
+      <c r="F67">
+        <v>699.38699999999994</v>
+      </c>
+      <c r="G67">
+        <f>SUM(D67:D72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>2036</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68">
+        <v>2</v>
+      </c>
+      <c r="D68">
+        <f t="shared" ref="D68:D72" si="11">E68*$F$69</f>
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>5.3561863952865569E-4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>2036</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69">
+        <v>3</v>
+      </c>
+      <c r="D69">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>0.27745045527584361</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>2036</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70">
+        <v>4</v>
+      </c>
+      <c r="D70">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>1.6604177825388325E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>2036</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71">
+        <v>5</v>
+      </c>
+      <c r="D71">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="E71">
+        <v>0.12961971076593465</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>2036</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72">
+        <v>6</v>
+      </c>
+      <c r="D72">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="E72">
+        <v>0.39903588644884846</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>